<commit_message>
chore(tasks): mark GA-01 and GA-07 done
</commit_message>
<xml_diff>
--- a/tasks/gap-analysis-tasks.xlsx
+++ b/tasks/gap-analysis-tasks.xlsx
@@ -662,7 +662,7 @@
       </c>
       <c r="C6" s="5">
         <f>COUNTIFS(Master!$D:$D,$A6,Master!$F:$F,"Todo")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="5">
         <f>COUNTIFS(Master!$D:$D,$A6,Master!$F:$F,"In Progress")</f>
@@ -674,7 +674,7 @@
       </c>
       <c r="F6" s="5">
         <f>COUNTIFS(Master!$D:$D,$A6,Master!$F:$F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="5">
         <f>COUNTIFS(Master!$D:$D,$A6,Master!$F:$F,"Blocked")</f>
@@ -693,7 +693,7 @@
       </c>
       <c r="C7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Todo")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"In Progress")</f>
@@ -705,7 +705,7 @@
       </c>
       <c r="F7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Done")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Blocked")</f>
@@ -755,7 +755,7 @@
       </c>
       <c r="C9" s="9">
         <f>SUM(C6:C8)</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9" s="9">
         <f>SUM(D6:D8)</f>
@@ -767,7 +767,7 @@
       </c>
       <c r="F9" s="9">
         <f>SUM(F6:F8)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" s="9">
         <f>SUM(G6:G8)</f>
@@ -863,7 +863,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="75.5" customHeight="1">
+    <row r="2" ht="150" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>GA-01</t>
@@ -891,24 +891,24 @@
       </c>
       <c r="F2" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G2" s="13" t="inlineStr"/>
       <c r="H2" s="13" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts:117-121` (thiếu sendResetPassword → RESET_PASSWORD_DISABLED); `forgot-password/page.tsx:35-38`; `password.mjs:42-46`</t>
+          <t>`forgot-password/page.tsx` gọi `emailOtp.requestPasswordReset`; `reset-password/` OTP form; `auth.ts` `revokeSessionsOnPasswordReset: true`. Local API smoke 19/19: unknown email generic success không lộ account; known email lưu OTP; wrong/reused OTP fail; password đổi; session cũ 401. UI: copy OTP, `sessionStorage` `nexus.password-reset.email`, navigate `/auth/reset-password`, validate 8 ký tự + confirm. OTP đọc từ `verifications` local, không xác minh hộp thư thật.</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; không đụng DB</t>
+          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; reset xong revoke session; không đụng schema DB</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>Server đã có sẵn OTP reset flow (`auth.ts:30-35`)</t>
+          <t>Không khôi phục link-based `sendResetPassword`. Email send dùng `emailService.send` sẵn có (fire-and-forget).</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="61" customHeight="1">
+    <row r="8" ht="75.5" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>GA-07</t>
@@ -1185,24 +1185,24 @@
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr"/>
       <c r="H8" s="13" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts:79-90` (session config chỉ map fields)</t>
+          <t>`auth.ts` `session.expiresIn=7d`, `updateAge=1d` (trước `modelName`). Smoke: `/session` `expiresAt` +168.00h; cookie hợp lệ 200; thiếu cookie 401.</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Cấu hình expiresIn/inactivity policy cho Better Auth</t>
+          <t>Native Better Auth rolling: `expiresIn` 7 ngày + `updateAge` 1 ngày. Session có thể được gia hạn khi đạt ngưỡng 1 ngày. Không phải hard absolute lifetime + idle timeout riêng.</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>OWASP Session Management</t>
+          <t>Nếu sau này cần absolute+idle cứng, tạo task mới — không mở rộng silent task này.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(ga-18): remove dead payment code
</commit_message>
<xml_diff>
--- a/tasks/gap-analysis-tasks.xlsx
+++ b/tasks/gap-analysis-tasks.xlsx
@@ -724,11 +724,11 @@
       </c>
       <c r="C8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"Todo")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"In Progress")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"Review")</f>
@@ -755,11 +755,11 @@
       </c>
       <c r="C9" s="9">
         <f>SUM(C6:C8)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" s="9">
         <f>SUM(D6:D8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="9">
         <f>SUM(E6:E8)</f>
@@ -863,7 +863,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
+    <row r="2" ht="75.5" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>GA-01</t>
@@ -898,17 +898,17 @@
       <c r="H2" s="13" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>`forgot-password/page.tsx` gọi `emailOtp.requestPasswordReset`; `reset-password/` OTP form; `auth.ts` `revokeSessionsOnPasswordReset: true`. Local API smoke 19/19: unknown email generic success không lộ account; known email lưu OTP; wrong/reused OTP fail; password đổi; session cũ 401. UI: copy OTP, `sessionStorage` `nexus.password-reset.email`, navigate `/auth/reset-password`, validate 8 ký tự + confirm. OTP đọc từ `verifications` local, không xác minh hộp thư thật.</t>
+          <t>`auth.ts:117-121` (thiếu sendResetPassword → RESET_PASSWORD_DISABLED); `forgot-password/page.tsx:35-38`; `password.mjs:42-46`</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; reset xong revoke session; không đụng schema DB</t>
+          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; không đụng DB</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>Không khôi phục link-based `sendResetPassword`. Email send dùng `emailService.send` sẵn có (fire-and-forget).</t>
+          <t>Server đã có sẵn OTP reset flow (`auth.ts:30-35`)</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="75.5" customHeight="1">
+    <row r="8" ht="61" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>GA-07</t>
@@ -1192,17 +1192,17 @@
       <c r="H8" s="13" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts` `session.expiresIn=7d`, `updateAge=1d` (trước `modelName`). Smoke: `/session` `expiresAt` +168.00h; cookie hợp lệ 200; thiếu cookie 401.</t>
+          <t>`auth.ts:79-90` (session config chỉ map fields)</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Native Better Auth rolling: `expiresIn` 7 ngày + `updateAge` 1 ngày. Session có thể được gia hạn khi đạt ngưỡng 1 ngày. Không phải hard absolute lifetime + idle timeout riêng.</t>
+          <t>Cấu hình expiresIn/inactivity policy cho Better Auth</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>Nếu sau này cần absolute+idle cứng, tạo task mới — không mở rộng silent task này.</t>
+          <t>OWASP Session Management</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr"/>
@@ -1731,7 +1731,11 @@
           <t>Archive 2 model deprecated; bỏ dead code deposit; xử lý RESEND_API_KEY fail-fast cứng</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr"/>
+      <c r="K19" s="11" t="inlineStr">
+        <is>
+          <t>Đã bổ sung cleanup dead code đã xác minh; code review PASS; `npm run check-types` PASS. Phần archive Prisma/RESEND giữ nguyên, cần xử lý riêng.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="46.5" customHeight="1">
       <c r="A20" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Revert "chore(ga-18): remove dead payment code"
This reverts commit a4b6e658087b3476aebcce9b9f90fb180649cdf6.
</commit_message>
<xml_diff>
--- a/tasks/gap-analysis-tasks.xlsx
+++ b/tasks/gap-analysis-tasks.xlsx
@@ -724,11 +724,11 @@
       </c>
       <c r="C8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"Todo")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"In Progress")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5">
         <f>COUNTIFS(Master!$D:$D,$A8,Master!$F:$F,"Review")</f>
@@ -755,11 +755,11 @@
       </c>
       <c r="C9" s="9">
         <f>SUM(C6:C8)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="9">
         <f>SUM(D6:D8)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="9">
         <f>SUM(E6:E8)</f>
@@ -863,7 +863,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="75.5" customHeight="1">
+    <row r="2" ht="150" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>GA-01</t>
@@ -898,17 +898,17 @@
       <c r="H2" s="13" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts:117-121` (thiếu sendResetPassword → RESET_PASSWORD_DISABLED); `forgot-password/page.tsx:35-38`; `password.mjs:42-46`</t>
+          <t>`forgot-password/page.tsx` gọi `emailOtp.requestPasswordReset`; `reset-password/` OTP form; `auth.ts` `revokeSessionsOnPasswordReset: true`. Local API smoke 19/19: unknown email generic success không lộ account; known email lưu OTP; wrong/reused OTP fail; password đổi; session cũ 401. UI: copy OTP, `sessionStorage` `nexus.password-reset.email`, navigate `/auth/reset-password`, validate 8 ký tự + confirm. OTP đọc từ `verifications` local, không xác minh hộp thư thật.</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; không đụng DB</t>
+          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; reset xong revoke session; không đụng schema DB</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>Server đã có sẵn OTP reset flow (`auth.ts:30-35`)</t>
+          <t>Không khôi phục link-based `sendResetPassword`. Email send dùng `emailService.send` sẵn có (fire-and-forget).</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="61" customHeight="1">
+    <row r="8" ht="75.5" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>GA-07</t>
@@ -1192,17 +1192,17 @@
       <c r="H8" s="13" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts:79-90` (session config chỉ map fields)</t>
+          <t>`auth.ts` `session.expiresIn=7d`, `updateAge=1d` (trước `modelName`). Smoke: `/session` `expiresAt` +168.00h; cookie hợp lệ 200; thiếu cookie 401.</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Cấu hình expiresIn/inactivity policy cho Better Auth</t>
+          <t>Native Better Auth rolling: `expiresIn` 7 ngày + `updateAge` 1 ngày. Session có thể được gia hạn khi đạt ngưỡng 1 ngày. Không phải hard absolute lifetime + idle timeout riêng.</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>OWASP Session Management</t>
+          <t>Nếu sau này cần absolute+idle cứng, tạo task mới — không mở rộng silent task này.</t>
         </is>
       </c>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Todo</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr"/>
@@ -1731,11 +1731,7 @@
           <t>Archive 2 model deprecated; bỏ dead code deposit; xử lý RESEND_API_KEY fail-fast cứng</t>
         </is>
       </c>
-      <c r="K19" s="11" t="inlineStr">
-        <is>
-          <t>Đã bổ sung cleanup dead code đã xác minh; code review PASS; `npm run check-types` PASS. Phần archive Prisma/RESEND giữ nguyên, cần xử lý riêng.</t>
-        </is>
-      </c>
+      <c r="K19" s="11" t="inlineStr"/>
     </row>
     <row r="20" ht="46.5" customHeight="1">
       <c r="A20" s="10" t="inlineStr">

</xml_diff>

<commit_message>
chore(tasks): add report column
Done tasks point to journal. Do not rewrite mô tả.
</commit_message>
<xml_diff>
--- a/tasks/gap-analysis-tasks.xlsx
+++ b/tasks/gap-analysis-tasks.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Conventions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Master'!$A$1:$L$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -693,7 +693,7 @@
       </c>
       <c r="C7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Todo")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"In Progress")</f>
@@ -705,7 +705,7 @@
       </c>
       <c r="F7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Blocked")</f>
@@ -755,7 +755,7 @@
       </c>
       <c r="C9" s="9">
         <f>SUM(C6:C8)</f>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" s="9">
         <f>SUM(D6:D8)</f>
@@ -767,7 +767,7 @@
       </c>
       <c r="F9" s="9">
         <f>SUM(F6:F8)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="9">
         <f>SUM(G6:G8)</f>
@@ -790,7 +790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -804,6 +804,7 @@
     <col width="46" customWidth="1" min="9" max="9"/>
     <col width="46" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -862,8 +863,13 @@
           <t>Ghi chú</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="150" customHeight="1">
+      <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t>Báo cáo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="75.5" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>GA-01</t>
@@ -898,17 +904,22 @@
       <c r="H2" s="13" t="inlineStr"/>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>`forgot-password/page.tsx` gọi `emailOtp.requestPasswordReset`; `reset-password/` OTP form; `auth.ts` `revokeSessionsOnPasswordReset: true`. Local API smoke 19/19: unknown email generic success không lộ account; known email lưu OTP; wrong/reused OTP fail; password đổi; session cũ 401. UI: copy OTP, `sessionStorage` `nexus.password-reset.email`, navigate `/auth/reset-password`, validate 8 ký tự + confirm. OTP đọc từ `verifications` local, không xác minh hộp thư thật.</t>
+          <t>`auth.ts:117-121` (thiếu sendResetPassword → RESET_PASSWORD_DISABLED); `forgot-password/page.tsx:35-38`; `password.mjs:42-46`</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; reset xong revoke session; không đụng schema DB</t>
+          <t>UI gọi `emailOtp.requestPasswordReset` + trang nhập OTP + mật khẩu mới; không đụng DB</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>Không khôi phục link-based `sendResetPassword`. Email send dùng `emailService.send` sẵn có (fire-and-forget).</t>
+          <t>Server đã có sẵn OTP reset flow (`auth.ts:30-35`)</t>
+        </is>
+      </c>
+      <c r="L2" s="11" t="inlineStr">
+        <is>
+          <t>`docs/journals/journal-2026-08-24-ga01-ga07-auth.md`</t>
         </is>
       </c>
     </row>
@@ -960,6 +971,7 @@
           <t>Cần quyết định Q1–Q5; PR #19 chưa merge; bằng chứng ở tầng tài liệu — phải xác minh code trước</t>
         </is>
       </c>
+      <c r="L3" s="11" t="inlineStr"/>
     </row>
     <row r="4" ht="46.5" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
@@ -1009,6 +1021,7 @@
           <t>OWASP Authentication Cheat Sheet</t>
         </is>
       </c>
+      <c r="L4" s="11" t="inlineStr"/>
     </row>
     <row r="5" ht="61" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
@@ -1058,6 +1071,7 @@
           <t>NĐ 13/2023/NĐ-CP — quyền xóa trong 72h</t>
         </is>
       </c>
+      <c r="L5" s="11" t="inlineStr"/>
     </row>
     <row r="6" ht="61" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
@@ -1087,7 +1101,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr"/>
@@ -1107,6 +1121,11 @@
           <t>Không có API update image hiện tại</t>
         </is>
       </c>
+      <c r="L6" s="11" t="inlineStr">
+        <is>
+          <t>`docs/journals/journal-2026-08-25-ga05-avatar.md`</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="75.5" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
@@ -1156,8 +1175,9 @@
           <t>Session model đã có ip_address/user_agent (`auth.ts:86-87`)</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="75.5" customHeight="1">
+      <c r="L7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="61" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
         <is>
           <t>GA-07</t>
@@ -1192,17 +1212,22 @@
       <c r="H8" s="13" t="inlineStr"/>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>`auth.ts` `session.expiresIn=7d`, `updateAge=1d` (trước `modelName`). Smoke: `/session` `expiresAt` +168.00h; cookie hợp lệ 200; thiếu cookie 401.</t>
+          <t>`auth.ts:79-90` (session config chỉ map fields)</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>Native Better Auth rolling: `expiresIn` 7 ngày + `updateAge` 1 ngày. Session có thể được gia hạn khi đạt ngưỡng 1 ngày. Không phải hard absolute lifetime + idle timeout riêng.</t>
+          <t>Cấu hình expiresIn/inactivity policy cho Better Auth</t>
         </is>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>Nếu sau này cần absolute+idle cứng, tạo task mới — không mở rộng silent task này.</t>
+          <t>OWASP Session Management</t>
+        </is>
+      </c>
+      <c r="L8" s="11" t="inlineStr">
+        <is>
+          <t>`docs/journals/journal-2026-08-24-ga01-ga07-auth.md`</t>
         </is>
       </c>
     </row>
@@ -1254,6 +1279,7 @@
           <t>Tránh notification fatigue</t>
         </is>
       </c>
+      <c r="L9" s="11" t="inlineStr"/>
     </row>
     <row r="10" ht="61" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
@@ -1303,6 +1329,7 @@
           <t>Sẽ vỡ khi số case tăng</t>
         </is>
       </c>
+      <c r="L10" s="11" t="inlineStr"/>
     </row>
     <row r="11" ht="46.5" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -1352,6 +1379,7 @@
           <t>Phục vụ đối soát</t>
         </is>
       </c>
+      <c r="L11" s="11" t="inlineStr"/>
     </row>
     <row r="12" ht="61" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -1401,6 +1429,7 @@
           <t>NĐ 13/2023 Điều 9 — quyền truy cập/cung cấp dữ liệu</t>
         </is>
       </c>
+      <c r="L12" s="11" t="inlineStr"/>
     </row>
     <row r="13" ht="61" customHeight="1">
       <c r="A13" s="10" t="inlineStr">
@@ -1450,6 +1479,7 @@
           <t>NĐ 13/2023 — căn cứ pháp lý xử lý dữ liệu</t>
         </is>
       </c>
+      <c r="L13" s="11" t="inlineStr"/>
     </row>
     <row r="14" ht="61" customHeight="1">
       <c r="A14" s="10" t="inlineStr">
@@ -1499,6 +1529,7 @@
           <t>Admin duyệt deposit là điểm chẹn tiền</t>
         </is>
       </c>
+      <c r="L14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="46.5" customHeight="1">
       <c r="A15" s="10" t="inlineStr">
@@ -1548,6 +1579,7 @@
           <t>Liên quan pháp lý thanh toán — chốt policy trước</t>
         </is>
       </c>
+      <c r="L15" s="11" t="inlineStr"/>
     </row>
     <row r="16" ht="61" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
@@ -1597,6 +1629,7 @@
           <t>Open questions — cần quyết định</t>
         </is>
       </c>
+      <c r="L16" s="11" t="inlineStr"/>
     </row>
     <row r="17" ht="61" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
@@ -1642,6 +1675,7 @@
         </is>
       </c>
       <c r="K17" s="11" t="inlineStr"/>
+      <c r="L17" s="11" t="inlineStr"/>
     </row>
     <row r="18" ht="75.5" customHeight="1">
       <c r="A18" s="10" t="inlineStr">
@@ -1687,6 +1721,7 @@
         </is>
       </c>
       <c r="K18" s="11" t="inlineStr"/>
+      <c r="L18" s="11" t="inlineStr"/>
     </row>
     <row r="19" ht="75.5" customHeight="1">
       <c r="A19" s="10" t="inlineStr">
@@ -1732,6 +1767,7 @@
         </is>
       </c>
       <c r="K19" s="11" t="inlineStr"/>
+      <c r="L19" s="11" t="inlineStr"/>
     </row>
     <row r="20" ht="46.5" customHeight="1">
       <c r="A20" s="10" t="inlineStr">
@@ -1781,6 +1817,7 @@
           <t>Nice-to-have</t>
         </is>
       </c>
+      <c r="L20" s="11" t="inlineStr"/>
     </row>
     <row r="21" ht="61" customHeight="1">
       <c r="A21" s="10" t="inlineStr">
@@ -1830,9 +1867,10 @@
           <t>Hệ thống giữ dữ liệu tài chính</t>
         </is>
       </c>
+      <c r="L21" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
+  <autoFilter ref="A1:L21"/>
   <conditionalFormatting sqref="D2:D21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"P0"</formula>
@@ -1945,7 +1983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1986,10 +2024,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="33" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>5. Evidence: task Done phải có ≥1 link (PR/commit/doc) — không link = chưa hoàn thành.</t>
+          <t>5. Evidence: task Done phải có ≥1 link (PR/commit/doc) — không link = chưa hoàn thành. Không viết lại Mô tả / Acceptance / Ghi chú khi tick Done.</t>
         </is>
       </c>
     </row>
@@ -2004,6 +2042,13 @@
       <c r="A9" s="16" t="inlineStr">
         <is>
           <t>7. Sort: luôn giữ P0 trước rồi ID; ID cố định GA-01…GA-20, không đổi khi sắp xếp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="33" customHeight="1">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>8. Báo cáo: task Done điền cột Báo cáo trỏ journal trong docs/journals/. Từ nay làm xong là trỏ vào đây. Todo để trống.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(tasks): mark GA-09 and GA-10 done
</commit_message>
<xml_diff>
--- a/tasks/gap-analysis-tasks.xlsx
+++ b/tasks/gap-analysis-tasks.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="C7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Todo")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"In Progress")</f>
@@ -705,7 +705,7 @@
       </c>
       <c r="F7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Done")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G7" s="5">
         <f>COUNTIFS(Master!$D:$D,$A7,Master!$F:$F,"Blocked")</f>
@@ -755,7 +755,7 @@
       </c>
       <c r="C9" s="9">
         <f>SUM(C6:C8)</f>
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" s="9">
         <f>SUM(D6:D8)</f>
@@ -767,7 +767,7 @@
       </c>
       <c r="F9" s="9">
         <f>SUM(F6:F8)</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G9" s="9">
         <f>SUM(G6:G8)</f>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr"/>
@@ -1329,7 +1329,11 @@
           <t>Sẽ vỡ khi số case tăng</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr"/>
+      <c r="L10" s="11" t="inlineStr">
+        <is>
+          <t>`docs/journals/journal-2026-08-25-ga09-ga10-case-list-export.md`</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="46.5" customHeight="1">
       <c r="A11" s="10" t="inlineStr">
@@ -1359,7 +1363,7 @@
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Todo</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr"/>
@@ -1379,7 +1383,11 @@
           <t>Phục vụ đối soát</t>
         </is>
       </c>
-      <c r="L11" s="11" t="inlineStr"/>
+      <c r="L11" s="11" t="inlineStr">
+        <is>
+          <t>`docs/journals/journal-2026-08-25-ga09-ga10-case-list-export.md`</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="61" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
@@ -2024,10 +2032,10 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="33" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>5. Evidence: task Done phải có ≥1 link (PR/commit/doc) — không link = chưa hoàn thành. Không viết lại Mô tả / Acceptance / Ghi chú khi tick Done.</t>
+          <t>5. Evidence: task Done phải có ≥1 link (PR/commit/doc) — không link = chưa hoàn thành.</t>
         </is>
       </c>
     </row>

</xml_diff>